<commit_message>
Deployed be2ef4d with MkDocs version: 1.6.1
</commit_message>
<xml_diff>
--- a/CIEL1/CCF/docs_officiels/repartition_annees.xlsx
+++ b/CIEL1/CCF/docs_officiels/repartition_annees.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\--- LYCEE ---\ENSEIGNEMENT_G\docs\CIEL1\CCF\docs_officiels\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5237D661-A40A-4C28-9DED-00DE5CAFB428}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E0D18924-BF14-4DA9-B2B3-5916061A55E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" activeTab="1" xr2:uid="{90326C7B-628B-4049-A4D0-57A32B541A41}"/>
+    <workbookView xWindow="10718" yWindow="0" windowWidth="10965" windowHeight="12863" activeTab="1" xr2:uid="{90326C7B-628B-4049-A4D0-57A32B541A41}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="456" uniqueCount="175">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="465" uniqueCount="184">
   <si>
     <t>Equa diff</t>
   </si>
@@ -284,9 +284,6 @@
     <t>Equations différentielles</t>
   </si>
   <si>
-    <t>Loi exponentielle</t>
-  </si>
-  <si>
     <t>Traitement du signal</t>
   </si>
   <si>
@@ -404,15 +401,9 @@
     <t>C216</t>
   </si>
   <si>
-    <t>TP Résolution Géogébra</t>
-  </si>
-  <si>
     <t>Loi de proba</t>
   </si>
   <si>
-    <t>Résolution par la calcul</t>
-  </si>
-  <si>
     <t>Résolution par Géogébra</t>
   </si>
   <si>
@@ -552,6 +543,42 @@
   </si>
   <si>
     <t>Loi binomiale</t>
+  </si>
+  <si>
+    <t>Lois continues</t>
+  </si>
+  <si>
+    <t>generalites</t>
+  </si>
+  <si>
+    <t>loi uniforme</t>
+  </si>
+  <si>
+    <t>loi normale</t>
+  </si>
+  <si>
+    <t>C227</t>
+  </si>
+  <si>
+    <t>C228</t>
+  </si>
+  <si>
+    <t>C229</t>
+  </si>
+  <si>
+    <t>TD lois continues</t>
+  </si>
+  <si>
+    <t>TP loi uniforme</t>
+  </si>
+  <si>
+    <t>TP loi normale</t>
+  </si>
+  <si>
+    <t>TP loi expo</t>
+  </si>
+  <si>
+    <t>loi exp</t>
   </si>
 </sst>
 </file>
@@ -2092,7 +2119,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{36FC5B6B-94BD-42C4-8F14-24F93C91EDDC}">
-  <dimension ref="A5:D66"/>
+  <dimension ref="A5:D72"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="2" max="2" width="30.06640625" customWidth="1"/>
@@ -2101,586 +2128,619 @@
   <sheetData>
     <row r="5" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B5" t="s">
         <v>84</v>
       </c>
       <c r="C5" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
       <c r="D5" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B6" t="s">
         <v>84</v>
       </c>
       <c r="C6" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="D6" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B7" t="s">
         <v>84</v>
       </c>
       <c r="C7" t="s">
+        <v>119</v>
+      </c>
+      <c r="D7" t="s">
         <v>120</v>
-      </c>
-      <c r="D7" t="s">
-        <v>121</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B8" t="s">
         <v>84</v>
       </c>
       <c r="C8" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="D8" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A9" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B9" t="s">
         <v>84</v>
       </c>
       <c r="C9" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="D9" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A10" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B10" t="s">
         <v>84</v>
       </c>
       <c r="C10" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="D10" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A11" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B11" t="s">
         <v>84</v>
       </c>
       <c r="C11" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="D11" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A12" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B12" t="s">
-        <v>85</v>
+        <v>172</v>
       </c>
       <c r="C12" t="s">
-        <v>119</v>
+        <v>173</v>
       </c>
       <c r="D12" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A13" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B13" t="s">
-        <v>85</v>
+        <v>172</v>
       </c>
       <c r="C13" t="s">
-        <v>126</v>
+        <v>174</v>
       </c>
       <c r="D13" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A14" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B14" t="s">
-        <v>85</v>
+        <v>172</v>
       </c>
       <c r="C14" t="s">
-        <v>127</v>
+        <v>175</v>
       </c>
       <c r="D14" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A15" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B15" t="s">
-        <v>85</v>
+        <v>172</v>
       </c>
       <c r="C15" t="s">
-        <v>128</v>
+        <v>183</v>
       </c>
       <c r="D15" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A16" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B16" t="s">
-        <v>85</v>
+        <v>172</v>
       </c>
       <c r="C16" t="s">
-        <v>125</v>
+        <v>179</v>
       </c>
       <c r="D16" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A17" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B17" t="s">
-        <v>85</v>
+        <v>172</v>
       </c>
       <c r="C17" t="s">
-        <v>125</v>
+        <v>180</v>
       </c>
       <c r="D17" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A18" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="B18" t="s">
-        <v>52</v>
+        <v>172</v>
       </c>
       <c r="C18" t="s">
-        <v>119</v>
+        <v>181</v>
       </c>
       <c r="D18" t="s">
-        <v>139</v>
+        <v>176</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A19" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="B19" t="s">
-        <v>52</v>
+        <v>172</v>
       </c>
       <c r="C19" t="s">
-        <v>126</v>
+        <v>182</v>
       </c>
       <c r="D19" t="s">
-        <v>140</v>
+        <v>177</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A20" t="s">
-        <v>96</v>
-      </c>
-      <c r="B20" t="s">
-        <v>52</v>
-      </c>
-      <c r="C20" t="s">
-        <v>134</v>
-      </c>
       <c r="D20" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A21" t="s">
-        <v>96</v>
-      </c>
-      <c r="B21" t="s">
-        <v>52</v>
-      </c>
-      <c r="C21" t="s">
-        <v>135</v>
-      </c>
-      <c r="D21" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A22" t="s">
-        <v>96</v>
-      </c>
-      <c r="B22" t="s">
-        <v>52</v>
-      </c>
-      <c r="C22" t="s">
-        <v>136</v>
-      </c>
-      <c r="D22" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A23" t="s">
-        <v>97</v>
-      </c>
-      <c r="B23" t="s">
-        <v>51</v>
-      </c>
-      <c r="C23" t="s">
-        <v>119</v>
-      </c>
-      <c r="D23" t="s">
-        <v>147</v>
+        <v>178</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A24" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="B24" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C24" t="s">
-        <v>126</v>
+        <v>118</v>
       </c>
       <c r="D24" t="s">
-        <v>148</v>
+        <v>136</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A25" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="B25" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C25" t="s">
-        <v>144</v>
+        <v>124</v>
       </c>
       <c r="D25" t="s">
-        <v>149</v>
+        <v>137</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A26" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="B26" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C26" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
       <c r="D26" t="s">
-        <v>150</v>
+        <v>138</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A27" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="B27" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C27" t="s">
-        <v>145</v>
+        <v>132</v>
       </c>
       <c r="D27" t="s">
-        <v>151</v>
+        <v>139</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A28" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="B28" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C28" t="s">
-        <v>146</v>
+        <v>133</v>
       </c>
       <c r="D28" t="s">
-        <v>152</v>
+        <v>140</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A29" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="B29" t="s">
-        <v>86</v>
+        <v>51</v>
       </c>
       <c r="C29" t="s">
-        <v>89</v>
+        <v>118</v>
       </c>
       <c r="D29" t="s">
-        <v>101</v>
+        <v>144</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A30" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="B30" t="s">
-        <v>86</v>
+        <v>51</v>
       </c>
       <c r="C30" t="s">
-        <v>90</v>
+        <v>124</v>
       </c>
       <c r="D30" t="s">
-        <v>102</v>
+        <v>145</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A31" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="B31" t="s">
-        <v>86</v>
+        <v>51</v>
       </c>
       <c r="C31" t="s">
-        <v>91</v>
+        <v>141</v>
       </c>
       <c r="D31" t="s">
-        <v>103</v>
+        <v>146</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A32" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="B32" t="s">
-        <v>86</v>
+        <v>51</v>
       </c>
       <c r="C32" t="s">
-        <v>92</v>
+        <v>125</v>
       </c>
       <c r="D32" t="s">
-        <v>104</v>
+        <v>147</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A33" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="B33" t="s">
-        <v>86</v>
+        <v>51</v>
       </c>
       <c r="C33" t="s">
-        <v>93</v>
+        <v>142</v>
       </c>
       <c r="D33" t="s">
-        <v>105</v>
+        <v>148</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A34" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="B34" t="s">
-        <v>86</v>
+        <v>51</v>
       </c>
       <c r="C34" t="s">
-        <v>106</v>
+        <v>143</v>
       </c>
       <c r="D34" t="s">
-        <v>110</v>
+        <v>149</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A35" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B35" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C35" t="s">
-        <v>107</v>
+        <v>88</v>
       </c>
       <c r="D35" t="s">
-        <v>111</v>
+        <v>100</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A36" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B36" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C36" t="s">
-        <v>108</v>
+        <v>89</v>
       </c>
       <c r="D36" t="s">
-        <v>112</v>
+        <v>101</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A37" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B37" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C37" t="s">
-        <v>109</v>
+        <v>90</v>
       </c>
       <c r="D37" t="s">
-        <v>113</v>
+        <v>102</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A38" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="B38" t="s">
-        <v>87</v>
+        <v>85</v>
+      </c>
+      <c r="C38" t="s">
+        <v>91</v>
+      </c>
+      <c r="D38" t="s">
+        <v>103</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A39" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="B39" t="s">
-        <v>88</v>
+        <v>85</v>
+      </c>
+      <c r="C39" t="s">
+        <v>92</v>
+      </c>
+      <c r="D39" t="s">
+        <v>104</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A40" t="s">
-        <v>114</v>
+        <v>97</v>
       </c>
       <c r="B40" t="s">
-        <v>39</v>
+        <v>85</v>
+      </c>
+      <c r="C40" t="s">
+        <v>105</v>
+      </c>
+      <c r="D40" t="s">
+        <v>109</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A41" t="s">
-        <v>115</v>
+        <v>97</v>
       </c>
       <c r="B41" t="s">
-        <v>116</v>
+        <v>85</v>
+      </c>
+      <c r="C41" t="s">
+        <v>106</v>
+      </c>
+      <c r="D41" t="s">
+        <v>110</v>
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A42" t="s">
+        <v>97</v>
+      </c>
       <c r="B42" t="s">
-        <v>70</v>
+        <v>85</v>
+      </c>
+      <c r="C42" t="s">
+        <v>107</v>
+      </c>
+      <c r="D42" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A43" t="s">
+        <v>97</v>
+      </c>
+      <c r="B43" t="s">
+        <v>85</v>
+      </c>
+      <c r="C43" t="s">
+        <v>108</v>
+      </c>
+      <c r="D43" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A44" t="s">
+        <v>98</v>
+      </c>
+      <c r="B44" t="s">
+        <v>86</v>
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A45" t="s">
-        <v>159</v>
+        <v>99</v>
       </c>
       <c r="B45" t="s">
-        <v>160</v>
-      </c>
-      <c r="C45" t="s">
-        <v>164</v>
+        <v>87</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A46" t="s">
+        <v>113</v>
+      </c>
+      <c r="B46" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A47" t="s">
+        <v>114</v>
+      </c>
+      <c r="B47" t="s">
+        <v>115</v>
       </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.45">
       <c r="B48" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="51" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A51" t="s">
+        <v>156</v>
+      </c>
+      <c r="B51" t="s">
+        <v>157</v>
+      </c>
+      <c r="C51" t="s">
         <v>161</v>
       </c>
-      <c r="C48" t="s">
+    </row>
+    <row r="54" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="B54" t="s">
+        <v>158</v>
+      </c>
+      <c r="C54" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="55" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="C55" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="56" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="C56" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="57" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="C57" t="s">
         <v>165</v>
       </c>
     </row>
-    <row r="49" spans="2:3" x14ac:dyDescent="0.45">
-      <c r="C49" t="s">
+    <row r="58" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="C58" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="59" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="C59" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="60" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="B60" t="s">
+        <v>2</v>
+      </c>
+      <c r="C60" t="s">
         <v>167</v>
       </c>
     </row>
-    <row r="50" spans="2:3" x14ac:dyDescent="0.45">
-      <c r="C50" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="51" spans="2:3" x14ac:dyDescent="0.45">
-      <c r="C51" t="s">
+    <row r="61" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="C61" t="s">
         <v>168</v>
       </c>
     </row>
-    <row r="52" spans="2:3" x14ac:dyDescent="0.45">
-      <c r="C52" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="53" spans="2:3" x14ac:dyDescent="0.45">
-      <c r="C53" t="s">
+    <row r="62" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="C62" t="s">
         <v>169</v>
       </c>
     </row>
-    <row r="54" spans="2:3" x14ac:dyDescent="0.45">
-      <c r="B54" t="s">
-        <v>2</v>
-      </c>
-      <c r="C54" t="s">
+    <row r="63" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="C63" t="s">
         <v>170</v>
       </c>
     </row>
-    <row r="55" spans="2:3" x14ac:dyDescent="0.45">
-      <c r="C55" t="s">
+    <row r="66" spans="2:3" x14ac:dyDescent="0.45">
+      <c r="B66" t="s">
+        <v>159</v>
+      </c>
+      <c r="C66" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="67" spans="2:3" x14ac:dyDescent="0.45">
+      <c r="C67" t="s">
         <v>171</v>
       </c>
     </row>
-    <row r="56" spans="2:3" x14ac:dyDescent="0.45">
-      <c r="C56" t="s">
-        <v>172</v>
-      </c>
-    </row>
-    <row r="57" spans="2:3" x14ac:dyDescent="0.45">
-      <c r="C57" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="60" spans="2:3" x14ac:dyDescent="0.45">
-      <c r="B60" t="s">
-        <v>162</v>
-      </c>
-      <c r="C60" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="61" spans="2:3" x14ac:dyDescent="0.45">
-      <c r="C61" t="s">
-        <v>174</v>
-      </c>
-    </row>
-    <row r="66" spans="2:2" x14ac:dyDescent="0.45">
-      <c r="B66" t="s">
-        <v>163</v>
+    <row r="72" spans="2:3" x14ac:dyDescent="0.45">
+      <c r="B72" t="s">
+        <v>160</v>
       </c>
     </row>
   </sheetData>

</xml_diff>